<commit_message>
fix: Prevent deletion of fee types with associated transactions and improve error handling in UI
</commit_message>
<xml_diff>
--- a/PMUAPI/database/seeders/PMU REPORT TEMPLATE.xlsx
+++ b/PMUAPI/database/seeders/PMU REPORT TEMPLATE.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Marthen Christ\source\repos\mccescario1995\PMU\PMUAPI\database\seeders\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{118D9183-6EFD-47A1-9FCB-3347D9890E06}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D71682B5-611D-46DD-882D-739B90EF34FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -272,18 +272,6 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="14" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
@@ -326,6 +314,18 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -334,6 +334,12 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="FFFFFF00"/>
+      <color rgb="FFFFFFFF"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -604,89 +610,89 @@
   </cols>
   <sheetData>
     <row r="11" spans="1:14" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="D11" s="6" t="s">
+      <c r="D11" s="23" t="s">
         <v>6</v>
       </c>
-      <c r="E11" s="6"/>
-      <c r="F11" s="6"/>
-      <c r="G11" s="6"/>
-      <c r="H11" s="6"/>
-      <c r="I11" s="6"/>
-      <c r="J11" s="6"/>
-      <c r="K11" s="6"/>
-      <c r="L11" s="6"/>
-      <c r="M11" s="6"/>
+      <c r="E11" s="23"/>
+      <c r="F11" s="23"/>
+      <c r="G11" s="23"/>
+      <c r="H11" s="23"/>
+      <c r="I11" s="23"/>
+      <c r="J11" s="23"/>
+      <c r="K11" s="23"/>
+      <c r="L11" s="23"/>
+      <c r="M11" s="23"/>
       <c r="N11" s="2"/>
     </row>
     <row r="13" spans="1:14" ht="29" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="19" t="s">
+      <c r="A13" s="15" t="s">
         <v>0</v>
       </c>
-      <c r="B13" s="26" t="s">
+      <c r="B13" s="22" t="s">
         <v>10</v>
       </c>
-      <c r="C13" s="20" t="s">
+      <c r="C13" s="16" t="s">
         <v>1</v>
       </c>
-      <c r="D13" s="10"/>
-      <c r="E13" s="11"/>
-      <c r="F13" s="12"/>
-      <c r="G13" s="13"/>
-      <c r="H13" s="14"/>
-      <c r="I13" s="11"/>
-      <c r="J13" s="11"/>
-      <c r="K13" s="11"/>
-      <c r="L13" s="15"/>
-      <c r="M13" s="14"/>
+      <c r="D13" s="6"/>
+      <c r="E13" s="7"/>
+      <c r="F13" s="8"/>
+      <c r="G13" s="9"/>
+      <c r="H13" s="10"/>
+      <c r="I13" s="7"/>
+      <c r="J13" s="7"/>
+      <c r="K13" s="7"/>
+      <c r="L13" s="11"/>
+      <c r="M13" s="10"/>
     </row>
     <row r="14" spans="1:14" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A14" s="23" t="s">
+      <c r="A14" s="19" t="s">
         <v>9</v>
       </c>
-      <c r="B14" s="25"/>
-      <c r="C14" s="21"/>
-      <c r="D14" s="13"/>
-      <c r="E14" s="11"/>
-      <c r="F14" s="13"/>
-      <c r="G14" s="12"/>
-      <c r="H14" s="11"/>
-      <c r="I14" s="11"/>
-      <c r="J14" s="11"/>
-      <c r="K14" s="11"/>
-      <c r="L14" s="11"/>
-      <c r="M14" s="11"/>
+      <c r="B14" s="21"/>
+      <c r="C14" s="17"/>
+      <c r="D14" s="9"/>
+      <c r="E14" s="7"/>
+      <c r="F14" s="9"/>
+      <c r="G14" s="8"/>
+      <c r="H14" s="7"/>
+      <c r="I14" s="7"/>
+      <c r="J14" s="7"/>
+      <c r="K14" s="7"/>
+      <c r="L14" s="7"/>
+      <c r="M14" s="7"/>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A15" s="24" t="s">
+      <c r="A15" s="20" t="s">
         <v>1</v>
       </c>
-      <c r="B15" s="22"/>
-      <c r="C15" s="22">
+      <c r="B15" s="18"/>
+      <c r="C15" s="18">
         <f>SUM(O16:O46)</f>
         <v>0</v>
       </c>
-      <c r="D15" s="16"/>
-      <c r="E15" s="16"/>
-      <c r="F15" s="16"/>
-      <c r="G15" s="16"/>
-      <c r="H15" s="17"/>
-      <c r="I15" s="16"/>
-      <c r="J15" s="16"/>
-      <c r="K15" s="16"/>
-      <c r="L15" s="16"/>
-      <c r="M15" s="16"/>
+      <c r="D15" s="12"/>
+      <c r="E15" s="12"/>
+      <c r="F15" s="12"/>
+      <c r="G15" s="12"/>
+      <c r="H15" s="13"/>
+      <c r="I15" s="12"/>
+      <c r="J15" s="12"/>
+      <c r="K15" s="12"/>
+      <c r="L15" s="12"/>
+      <c r="M15" s="12"/>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="D16" s="18"/>
-      <c r="E16" s="18"/>
-      <c r="F16" s="18"/>
-      <c r="G16" s="18"/>
-      <c r="H16" s="18"/>
-      <c r="I16" s="18"/>
-      <c r="J16" s="18"/>
-      <c r="K16" s="18"/>
-      <c r="L16" s="18"/>
-      <c r="M16" s="18"/>
+      <c r="D16" s="14"/>
+      <c r="E16" s="14"/>
+      <c r="F16" s="14"/>
+      <c r="G16" s="14"/>
+      <c r="H16" s="14"/>
+      <c r="I16" s="14"/>
+      <c r="J16" s="14"/>
+      <c r="K16" s="14"/>
+      <c r="L16" s="14"/>
+      <c r="M16" s="14"/>
     </row>
     <row r="18" spans="1:15" x14ac:dyDescent="0.35">
       <c r="B18" s="1" t="s">
@@ -697,432 +703,432 @@
       </c>
     </row>
     <row r="20" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="C20" s="5" t="s">
+      <c r="C20" s="26" t="s">
         <v>7</v>
       </c>
-      <c r="D20" s="5"/>
-      <c r="L20" s="3" t="s">
+      <c r="D20" s="26"/>
+      <c r="L20" s="24" t="s">
         <v>4</v>
       </c>
-      <c r="M20" s="3"/>
+      <c r="M20" s="24"/>
     </row>
     <row r="21" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="C21" s="4" t="s">
+      <c r="C21" s="25" t="s">
         <v>8</v>
       </c>
-      <c r="D21" s="4"/>
-      <c r="L21" s="4" t="s">
+      <c r="D21" s="25"/>
+      <c r="L21" s="25" t="s">
         <v>5</v>
       </c>
-      <c r="M21" s="4"/>
+      <c r="M21" s="25"/>
     </row>
     <row r="23" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A23" s="7"/>
-      <c r="B23" s="8"/>
-      <c r="C23" s="8"/>
-      <c r="D23" s="8"/>
-      <c r="E23" s="8"/>
-      <c r="F23" s="8"/>
-      <c r="G23" s="8"/>
-      <c r="H23" s="8"/>
-      <c r="I23" s="8"/>
-      <c r="J23" s="8"/>
-      <c r="K23" s="8"/>
-      <c r="L23" s="8"/>
-      <c r="M23" s="8"/>
-      <c r="N23" s="8"/>
-      <c r="O23" s="8"/>
+      <c r="A23" s="3"/>
+      <c r="B23" s="4"/>
+      <c r="C23" s="4"/>
+      <c r="D23" s="4"/>
+      <c r="E23" s="4"/>
+      <c r="F23" s="4"/>
+      <c r="G23" s="4"/>
+      <c r="H23" s="4"/>
+      <c r="I23" s="4"/>
+      <c r="J23" s="4"/>
+      <c r="K23" s="4"/>
+      <c r="L23" s="4"/>
+      <c r="M23" s="4"/>
+      <c r="N23" s="4"/>
+      <c r="O23" s="4"/>
     </row>
     <row r="24" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A24" s="7"/>
-      <c r="B24" s="8"/>
-      <c r="C24" s="8"/>
-      <c r="D24" s="8"/>
-      <c r="E24" s="8"/>
-      <c r="F24" s="8"/>
-      <c r="G24" s="8"/>
-      <c r="H24" s="8"/>
-      <c r="I24" s="8"/>
-      <c r="J24" s="8"/>
-      <c r="K24" s="8"/>
-      <c r="L24" s="8"/>
-      <c r="M24" s="8"/>
-      <c r="N24" s="8"/>
-      <c r="O24" s="8"/>
+      <c r="A24" s="3"/>
+      <c r="B24" s="4"/>
+      <c r="C24" s="4"/>
+      <c r="D24" s="4"/>
+      <c r="E24" s="4"/>
+      <c r="F24" s="4"/>
+      <c r="G24" s="4"/>
+      <c r="H24" s="4"/>
+      <c r="I24" s="4"/>
+      <c r="J24" s="4"/>
+      <c r="K24" s="4"/>
+      <c r="L24" s="4"/>
+      <c r="M24" s="4"/>
+      <c r="N24" s="4"/>
+      <c r="O24" s="4"/>
     </row>
     <row r="25" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A25" s="7"/>
-      <c r="B25" s="8"/>
-      <c r="C25" s="8"/>
-      <c r="D25" s="8"/>
-      <c r="E25" s="8"/>
-      <c r="F25" s="8"/>
-      <c r="G25" s="8"/>
-      <c r="H25" s="8"/>
-      <c r="I25" s="8"/>
-      <c r="J25" s="8"/>
-      <c r="K25" s="8"/>
-      <c r="L25" s="8"/>
-      <c r="M25" s="8"/>
-      <c r="N25" s="8"/>
-      <c r="O25" s="8"/>
+      <c r="A25" s="3"/>
+      <c r="B25" s="4"/>
+      <c r="C25" s="4"/>
+      <c r="D25" s="4"/>
+      <c r="E25" s="4"/>
+      <c r="F25" s="4"/>
+      <c r="G25" s="4"/>
+      <c r="H25" s="4"/>
+      <c r="I25" s="4"/>
+      <c r="J25" s="4"/>
+      <c r="K25" s="4"/>
+      <c r="L25" s="4"/>
+      <c r="M25" s="4"/>
+      <c r="N25" s="4"/>
+      <c r="O25" s="4"/>
     </row>
     <row r="26" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A26" s="7"/>
-      <c r="B26" s="8"/>
-      <c r="C26" s="8"/>
-      <c r="D26" s="8"/>
-      <c r="E26" s="8"/>
-      <c r="F26" s="8"/>
-      <c r="G26" s="8"/>
-      <c r="H26" s="8"/>
-      <c r="I26" s="8"/>
-      <c r="J26" s="8"/>
-      <c r="K26" s="8"/>
-      <c r="L26" s="8"/>
-      <c r="M26" s="8"/>
-      <c r="N26" s="8"/>
-      <c r="O26" s="8"/>
+      <c r="A26" s="3"/>
+      <c r="B26" s="4"/>
+      <c r="C26" s="4"/>
+      <c r="D26" s="4"/>
+      <c r="E26" s="4"/>
+      <c r="F26" s="4"/>
+      <c r="G26" s="4"/>
+      <c r="H26" s="4"/>
+      <c r="I26" s="4"/>
+      <c r="J26" s="4"/>
+      <c r="K26" s="4"/>
+      <c r="L26" s="4"/>
+      <c r="M26" s="4"/>
+      <c r="N26" s="4"/>
+      <c r="O26" s="4"/>
     </row>
     <row r="27" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A27" s="7"/>
-      <c r="B27" s="8"/>
-      <c r="C27" s="8"/>
-      <c r="D27" s="8"/>
-      <c r="E27" s="8"/>
-      <c r="F27" s="8"/>
-      <c r="G27" s="8"/>
-      <c r="H27" s="8"/>
-      <c r="I27" s="8"/>
-      <c r="J27" s="8"/>
-      <c r="K27" s="8"/>
-      <c r="L27" s="8"/>
-      <c r="M27" s="8"/>
-      <c r="N27" s="8"/>
-      <c r="O27" s="8"/>
+      <c r="A27" s="3"/>
+      <c r="B27" s="4"/>
+      <c r="C27" s="4"/>
+      <c r="D27" s="4"/>
+      <c r="E27" s="4"/>
+      <c r="F27" s="4"/>
+      <c r="G27" s="4"/>
+      <c r="H27" s="4"/>
+      <c r="I27" s="4"/>
+      <c r="J27" s="4"/>
+      <c r="K27" s="4"/>
+      <c r="L27" s="4"/>
+      <c r="M27" s="4"/>
+      <c r="N27" s="4"/>
+      <c r="O27" s="4"/>
     </row>
     <row r="28" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A28" s="7"/>
-      <c r="B28" s="8"/>
-      <c r="C28" s="8"/>
-      <c r="D28" s="8"/>
-      <c r="E28" s="8"/>
-      <c r="F28" s="8"/>
-      <c r="G28" s="8"/>
-      <c r="H28" s="8"/>
-      <c r="I28" s="8"/>
-      <c r="J28" s="8"/>
-      <c r="K28" s="8"/>
-      <c r="L28" s="8"/>
-      <c r="M28" s="8"/>
-      <c r="N28" s="8"/>
-      <c r="O28" s="8"/>
+      <c r="A28" s="3"/>
+      <c r="B28" s="4"/>
+      <c r="C28" s="4"/>
+      <c r="D28" s="4"/>
+      <c r="E28" s="4"/>
+      <c r="F28" s="4"/>
+      <c r="G28" s="4"/>
+      <c r="H28" s="4"/>
+      <c r="I28" s="4"/>
+      <c r="J28" s="4"/>
+      <c r="K28" s="4"/>
+      <c r="L28" s="4"/>
+      <c r="M28" s="4"/>
+      <c r="N28" s="4"/>
+      <c r="O28" s="4"/>
     </row>
     <row r="29" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A29" s="7"/>
-      <c r="B29" s="8"/>
-      <c r="C29" s="8"/>
-      <c r="D29" s="8"/>
-      <c r="E29" s="8"/>
-      <c r="F29" s="8"/>
-      <c r="G29" s="8"/>
-      <c r="H29" s="8"/>
-      <c r="I29" s="8"/>
-      <c r="J29" s="8"/>
-      <c r="K29" s="8"/>
-      <c r="L29" s="8"/>
-      <c r="M29" s="8"/>
-      <c r="N29" s="8"/>
-      <c r="O29" s="8"/>
+      <c r="A29" s="3"/>
+      <c r="B29" s="4"/>
+      <c r="C29" s="4"/>
+      <c r="D29" s="4"/>
+      <c r="E29" s="4"/>
+      <c r="F29" s="4"/>
+      <c r="G29" s="4"/>
+      <c r="H29" s="4"/>
+      <c r="I29" s="4"/>
+      <c r="J29" s="4"/>
+      <c r="K29" s="4"/>
+      <c r="L29" s="4"/>
+      <c r="M29" s="4"/>
+      <c r="N29" s="4"/>
+      <c r="O29" s="4"/>
     </row>
     <row r="30" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A30" s="7"/>
-      <c r="B30" s="8"/>
-      <c r="C30" s="8"/>
-      <c r="D30" s="8"/>
-      <c r="E30" s="8"/>
-      <c r="F30" s="8"/>
-      <c r="G30" s="8"/>
-      <c r="H30" s="8"/>
-      <c r="I30" s="8"/>
-      <c r="J30" s="8"/>
-      <c r="K30" s="8"/>
-      <c r="L30" s="8"/>
-      <c r="M30" s="8"/>
-      <c r="N30" s="8"/>
-      <c r="O30" s="8"/>
+      <c r="A30" s="3"/>
+      <c r="B30" s="4"/>
+      <c r="C30" s="4"/>
+      <c r="D30" s="4"/>
+      <c r="E30" s="4"/>
+      <c r="F30" s="4"/>
+      <c r="G30" s="4"/>
+      <c r="H30" s="4"/>
+      <c r="I30" s="4"/>
+      <c r="J30" s="4"/>
+      <c r="K30" s="4"/>
+      <c r="L30" s="4"/>
+      <c r="M30" s="4"/>
+      <c r="N30" s="4"/>
+      <c r="O30" s="4"/>
     </row>
     <row r="31" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A31" s="7"/>
-      <c r="B31" s="8"/>
-      <c r="C31" s="8"/>
-      <c r="D31" s="8"/>
-      <c r="E31" s="8"/>
-      <c r="F31" s="8"/>
-      <c r="G31" s="8"/>
-      <c r="H31" s="8"/>
-      <c r="I31" s="8"/>
-      <c r="J31" s="8"/>
-      <c r="K31" s="8"/>
-      <c r="L31" s="8"/>
-      <c r="M31" s="8"/>
-      <c r="N31" s="8"/>
-      <c r="O31" s="8"/>
+      <c r="A31" s="3"/>
+      <c r="B31" s="4"/>
+      <c r="C31" s="4"/>
+      <c r="D31" s="4"/>
+      <c r="E31" s="4"/>
+      <c r="F31" s="4"/>
+      <c r="G31" s="4"/>
+      <c r="H31" s="4"/>
+      <c r="I31" s="4"/>
+      <c r="J31" s="4"/>
+      <c r="K31" s="4"/>
+      <c r="L31" s="4"/>
+      <c r="M31" s="4"/>
+      <c r="N31" s="4"/>
+      <c r="O31" s="4"/>
     </row>
     <row r="32" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A32" s="7"/>
-      <c r="B32" s="8"/>
-      <c r="C32" s="8"/>
-      <c r="D32" s="8"/>
-      <c r="E32" s="8"/>
-      <c r="F32" s="8"/>
-      <c r="G32" s="8"/>
-      <c r="H32" s="8"/>
-      <c r="I32" s="8"/>
-      <c r="J32" s="8"/>
-      <c r="K32" s="8"/>
-      <c r="L32" s="8"/>
-      <c r="M32" s="8"/>
-      <c r="N32" s="8"/>
-      <c r="O32" s="8"/>
+      <c r="A32" s="3"/>
+      <c r="B32" s="4"/>
+      <c r="C32" s="4"/>
+      <c r="D32" s="4"/>
+      <c r="E32" s="4"/>
+      <c r="F32" s="4"/>
+      <c r="G32" s="4"/>
+      <c r="H32" s="4"/>
+      <c r="I32" s="4"/>
+      <c r="J32" s="4"/>
+      <c r="K32" s="4"/>
+      <c r="L32" s="4"/>
+      <c r="M32" s="4"/>
+      <c r="N32" s="4"/>
+      <c r="O32" s="4"/>
     </row>
     <row r="33" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A33" s="7"/>
-      <c r="B33" s="8"/>
-      <c r="C33" s="8"/>
-      <c r="D33" s="8"/>
-      <c r="E33" s="8"/>
-      <c r="F33" s="8"/>
-      <c r="G33" s="8"/>
-      <c r="H33" s="8"/>
-      <c r="I33" s="8"/>
-      <c r="J33" s="8"/>
-      <c r="K33" s="8"/>
-      <c r="L33" s="8"/>
-      <c r="M33" s="8"/>
-      <c r="N33" s="8"/>
-      <c r="O33" s="8"/>
+      <c r="A33" s="3"/>
+      <c r="B33" s="4"/>
+      <c r="C33" s="4"/>
+      <c r="D33" s="4"/>
+      <c r="E33" s="4"/>
+      <c r="F33" s="4"/>
+      <c r="G33" s="4"/>
+      <c r="H33" s="4"/>
+      <c r="I33" s="4"/>
+      <c r="J33" s="4"/>
+      <c r="K33" s="4"/>
+      <c r="L33" s="4"/>
+      <c r="M33" s="4"/>
+      <c r="N33" s="4"/>
+      <c r="O33" s="4"/>
     </row>
     <row r="34" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A34" s="7"/>
-      <c r="B34" s="8"/>
-      <c r="C34" s="8"/>
-      <c r="D34" s="8"/>
-      <c r="E34" s="8"/>
-      <c r="F34" s="8"/>
-      <c r="G34" s="8"/>
-      <c r="H34" s="8"/>
-      <c r="I34" s="8"/>
-      <c r="J34" s="8"/>
-      <c r="K34" s="8"/>
-      <c r="L34" s="8"/>
-      <c r="M34" s="8"/>
-      <c r="N34" s="8"/>
-      <c r="O34" s="8"/>
+      <c r="A34" s="3"/>
+      <c r="B34" s="4"/>
+      <c r="C34" s="4"/>
+      <c r="D34" s="4"/>
+      <c r="E34" s="4"/>
+      <c r="F34" s="4"/>
+      <c r="G34" s="4"/>
+      <c r="H34" s="4"/>
+      <c r="I34" s="4"/>
+      <c r="J34" s="4"/>
+      <c r="K34" s="4"/>
+      <c r="L34" s="4"/>
+      <c r="M34" s="4"/>
+      <c r="N34" s="4"/>
+      <c r="O34" s="4"/>
     </row>
     <row r="35" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A35" s="7"/>
-      <c r="B35" s="8"/>
-      <c r="C35" s="8"/>
-      <c r="D35" s="8"/>
-      <c r="E35" s="8"/>
-      <c r="F35" s="8"/>
-      <c r="G35" s="8"/>
-      <c r="H35" s="8"/>
-      <c r="I35" s="8"/>
-      <c r="J35" s="8"/>
-      <c r="K35" s="8"/>
-      <c r="L35" s="8"/>
-      <c r="M35" s="8"/>
-      <c r="N35" s="8"/>
-      <c r="O35" s="8"/>
+      <c r="A35" s="3"/>
+      <c r="B35" s="4"/>
+      <c r="C35" s="4"/>
+      <c r="D35" s="4"/>
+      <c r="E35" s="4"/>
+      <c r="F35" s="4"/>
+      <c r="G35" s="4"/>
+      <c r="H35" s="4"/>
+      <c r="I35" s="4"/>
+      <c r="J35" s="4"/>
+      <c r="K35" s="4"/>
+      <c r="L35" s="4"/>
+      <c r="M35" s="4"/>
+      <c r="N35" s="4"/>
+      <c r="O35" s="4"/>
     </row>
     <row r="36" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A36" s="7"/>
-      <c r="B36" s="8"/>
-      <c r="C36" s="8"/>
-      <c r="D36" s="8"/>
-      <c r="E36" s="8"/>
-      <c r="F36" s="8"/>
-      <c r="G36" s="8"/>
-      <c r="H36" s="8"/>
-      <c r="I36" s="8"/>
-      <c r="J36" s="8"/>
-      <c r="K36" s="8"/>
-      <c r="L36" s="8"/>
-      <c r="M36" s="8"/>
-      <c r="N36" s="8"/>
-      <c r="O36" s="8"/>
+      <c r="A36" s="3"/>
+      <c r="B36" s="4"/>
+      <c r="C36" s="4"/>
+      <c r="D36" s="4"/>
+      <c r="E36" s="4"/>
+      <c r="F36" s="4"/>
+      <c r="G36" s="4"/>
+      <c r="H36" s="4"/>
+      <c r="I36" s="4"/>
+      <c r="J36" s="4"/>
+      <c r="K36" s="4"/>
+      <c r="L36" s="4"/>
+      <c r="M36" s="4"/>
+      <c r="N36" s="4"/>
+      <c r="O36" s="4"/>
     </row>
     <row r="37" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A37" s="7"/>
-      <c r="B37" s="8"/>
-      <c r="C37" s="8"/>
-      <c r="D37" s="8"/>
-      <c r="E37" s="8"/>
-      <c r="F37" s="8"/>
-      <c r="G37" s="8"/>
-      <c r="H37" s="8"/>
-      <c r="I37" s="8"/>
-      <c r="J37" s="8"/>
-      <c r="K37" s="8"/>
-      <c r="L37" s="8"/>
-      <c r="M37" s="8"/>
-      <c r="N37" s="8"/>
-      <c r="O37" s="8"/>
+      <c r="A37" s="3"/>
+      <c r="B37" s="4"/>
+      <c r="C37" s="4"/>
+      <c r="D37" s="4"/>
+      <c r="E37" s="4"/>
+      <c r="F37" s="4"/>
+      <c r="G37" s="4"/>
+      <c r="H37" s="4"/>
+      <c r="I37" s="4"/>
+      <c r="J37" s="4"/>
+      <c r="K37" s="4"/>
+      <c r="L37" s="4"/>
+      <c r="M37" s="4"/>
+      <c r="N37" s="4"/>
+      <c r="O37" s="4"/>
     </row>
     <row r="38" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A38" s="7"/>
-      <c r="B38" s="8"/>
-      <c r="C38" s="8"/>
-      <c r="D38" s="8"/>
-      <c r="E38" s="8"/>
-      <c r="F38" s="8"/>
-      <c r="G38" s="8"/>
-      <c r="H38" s="8"/>
-      <c r="I38" s="8"/>
-      <c r="J38" s="8"/>
-      <c r="K38" s="8"/>
-      <c r="L38" s="8"/>
-      <c r="M38" s="8"/>
-      <c r="N38" s="8"/>
-      <c r="O38" s="8"/>
+      <c r="A38" s="3"/>
+      <c r="B38" s="4"/>
+      <c r="C38" s="4"/>
+      <c r="D38" s="4"/>
+      <c r="E38" s="4"/>
+      <c r="F38" s="4"/>
+      <c r="G38" s="4"/>
+      <c r="H38" s="4"/>
+      <c r="I38" s="4"/>
+      <c r="J38" s="4"/>
+      <c r="K38" s="4"/>
+      <c r="L38" s="4"/>
+      <c r="M38" s="4"/>
+      <c r="N38" s="4"/>
+      <c r="O38" s="4"/>
     </row>
     <row r="39" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A39" s="7"/>
-      <c r="B39" s="8"/>
-      <c r="C39" s="8"/>
-      <c r="D39" s="8"/>
-      <c r="E39" s="8"/>
-      <c r="F39" s="8"/>
-      <c r="G39" s="8"/>
-      <c r="H39" s="8"/>
-      <c r="I39" s="8"/>
-      <c r="J39" s="8"/>
-      <c r="K39" s="8"/>
-      <c r="L39" s="8"/>
-      <c r="M39" s="8"/>
-      <c r="N39" s="8"/>
-      <c r="O39" s="8"/>
+      <c r="A39" s="3"/>
+      <c r="B39" s="4"/>
+      <c r="C39" s="4"/>
+      <c r="D39" s="4"/>
+      <c r="E39" s="4"/>
+      <c r="F39" s="4"/>
+      <c r="G39" s="4"/>
+      <c r="H39" s="4"/>
+      <c r="I39" s="4"/>
+      <c r="J39" s="4"/>
+      <c r="K39" s="4"/>
+      <c r="L39" s="4"/>
+      <c r="M39" s="4"/>
+      <c r="N39" s="4"/>
+      <c r="O39" s="4"/>
     </row>
     <row r="40" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A40" s="7"/>
-      <c r="B40" s="8"/>
-      <c r="C40" s="8"/>
-      <c r="D40" s="8"/>
-      <c r="E40" s="8"/>
-      <c r="F40" s="8"/>
-      <c r="G40" s="8"/>
-      <c r="H40" s="8"/>
-      <c r="I40" s="8"/>
-      <c r="J40" s="8"/>
-      <c r="K40" s="8"/>
-      <c r="L40" s="8"/>
-      <c r="M40" s="8"/>
-      <c r="N40" s="8"/>
-      <c r="O40" s="8"/>
+      <c r="A40" s="3"/>
+      <c r="B40" s="4"/>
+      <c r="C40" s="4"/>
+      <c r="D40" s="4"/>
+      <c r="E40" s="4"/>
+      <c r="F40" s="4"/>
+      <c r="G40" s="4"/>
+      <c r="H40" s="4"/>
+      <c r="I40" s="4"/>
+      <c r="J40" s="4"/>
+      <c r="K40" s="4"/>
+      <c r="L40" s="4"/>
+      <c r="M40" s="4"/>
+      <c r="N40" s="4"/>
+      <c r="O40" s="4"/>
     </row>
     <row r="41" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A41" s="7"/>
-      <c r="B41" s="8"/>
-      <c r="C41" s="8"/>
-      <c r="D41" s="8"/>
-      <c r="E41" s="8"/>
-      <c r="F41" s="8"/>
-      <c r="G41" s="8"/>
-      <c r="H41" s="8"/>
-      <c r="I41" s="8"/>
-      <c r="J41" s="8"/>
-      <c r="K41" s="8"/>
-      <c r="L41" s="8"/>
-      <c r="M41" s="8"/>
-      <c r="N41" s="8"/>
-      <c r="O41" s="8"/>
+      <c r="A41" s="3"/>
+      <c r="B41" s="4"/>
+      <c r="C41" s="4"/>
+      <c r="D41" s="4"/>
+      <c r="E41" s="4"/>
+      <c r="F41" s="4"/>
+      <c r="G41" s="4"/>
+      <c r="H41" s="4"/>
+      <c r="I41" s="4"/>
+      <c r="J41" s="4"/>
+      <c r="K41" s="4"/>
+      <c r="L41" s="4"/>
+      <c r="M41" s="4"/>
+      <c r="N41" s="4"/>
+      <c r="O41" s="4"/>
     </row>
     <row r="42" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A42" s="7"/>
-      <c r="B42" s="8"/>
-      <c r="C42" s="8"/>
-      <c r="D42" s="8"/>
-      <c r="E42" s="8"/>
-      <c r="F42" s="8"/>
-      <c r="G42" s="8"/>
-      <c r="H42" s="8"/>
-      <c r="I42" s="8"/>
-      <c r="J42" s="8"/>
-      <c r="K42" s="8"/>
-      <c r="L42" s="8"/>
-      <c r="M42" s="8"/>
-      <c r="N42" s="8"/>
-      <c r="O42" s="8"/>
+      <c r="A42" s="3"/>
+      <c r="B42" s="4"/>
+      <c r="C42" s="4"/>
+      <c r="D42" s="4"/>
+      <c r="E42" s="4"/>
+      <c r="F42" s="4"/>
+      <c r="G42" s="4"/>
+      <c r="H42" s="4"/>
+      <c r="I42" s="4"/>
+      <c r="J42" s="4"/>
+      <c r="K42" s="4"/>
+      <c r="L42" s="4"/>
+      <c r="M42" s="4"/>
+      <c r="N42" s="4"/>
+      <c r="O42" s="4"/>
     </row>
     <row r="43" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A43" s="7"/>
-      <c r="B43" s="8"/>
-      <c r="C43" s="8"/>
-      <c r="D43" s="8"/>
-      <c r="E43" s="8"/>
-      <c r="F43" s="8"/>
-      <c r="G43" s="8"/>
-      <c r="H43" s="8"/>
-      <c r="I43" s="8"/>
-      <c r="J43" s="8"/>
-      <c r="K43" s="8"/>
-      <c r="L43" s="8"/>
-      <c r="M43" s="9"/>
-      <c r="N43" s="8"/>
-      <c r="O43" s="8"/>
+      <c r="A43" s="3"/>
+      <c r="B43" s="4"/>
+      <c r="C43" s="4"/>
+      <c r="D43" s="4"/>
+      <c r="E43" s="4"/>
+      <c r="F43" s="4"/>
+      <c r="G43" s="4"/>
+      <c r="H43" s="4"/>
+      <c r="I43" s="4"/>
+      <c r="J43" s="4"/>
+      <c r="K43" s="4"/>
+      <c r="L43" s="4"/>
+      <c r="M43" s="5"/>
+      <c r="N43" s="4"/>
+      <c r="O43" s="4"/>
     </row>
     <row r="44" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A44" s="7"/>
-      <c r="B44" s="8"/>
-      <c r="C44" s="8"/>
-      <c r="D44" s="8"/>
-      <c r="E44" s="8"/>
-      <c r="F44" s="8"/>
-      <c r="G44" s="8"/>
-      <c r="H44" s="8"/>
-      <c r="I44" s="8"/>
-      <c r="J44" s="8"/>
-      <c r="K44" s="8"/>
-      <c r="L44" s="8"/>
-      <c r="M44" s="8"/>
-      <c r="N44" s="8"/>
-      <c r="O44" s="8"/>
+      <c r="A44" s="3"/>
+      <c r="B44" s="4"/>
+      <c r="C44" s="4"/>
+      <c r="D44" s="4"/>
+      <c r="E44" s="4"/>
+      <c r="F44" s="4"/>
+      <c r="G44" s="4"/>
+      <c r="H44" s="4"/>
+      <c r="I44" s="4"/>
+      <c r="J44" s="4"/>
+      <c r="K44" s="4"/>
+      <c r="L44" s="4"/>
+      <c r="M44" s="4"/>
+      <c r="N44" s="4"/>
+      <c r="O44" s="4"/>
     </row>
     <row r="45" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A45" s="7"/>
-      <c r="B45" s="8"/>
-      <c r="C45" s="8"/>
-      <c r="D45" s="8"/>
-      <c r="E45" s="8"/>
-      <c r="F45" s="8"/>
-      <c r="G45" s="8"/>
-      <c r="H45" s="8"/>
-      <c r="I45" s="8"/>
-      <c r="J45" s="8"/>
-      <c r="K45" s="8"/>
-      <c r="L45" s="8"/>
-      <c r="M45" s="8"/>
-      <c r="N45" s="8"/>
-      <c r="O45" s="8"/>
+      <c r="A45" s="3"/>
+      <c r="B45" s="4"/>
+      <c r="C45" s="4"/>
+      <c r="D45" s="4"/>
+      <c r="E45" s="4"/>
+      <c r="F45" s="4"/>
+      <c r="G45" s="4"/>
+      <c r="H45" s="4"/>
+      <c r="I45" s="4"/>
+      <c r="J45" s="4"/>
+      <c r="K45" s="4"/>
+      <c r="L45" s="4"/>
+      <c r="M45" s="4"/>
+      <c r="N45" s="4"/>
+      <c r="O45" s="4"/>
     </row>
     <row r="46" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A46" s="7"/>
-      <c r="B46" s="8"/>
-      <c r="C46" s="8"/>
-      <c r="D46" s="8"/>
-      <c r="E46" s="8"/>
-      <c r="F46" s="8"/>
-      <c r="G46" s="8"/>
-      <c r="H46" s="8"/>
-      <c r="I46" s="8"/>
-      <c r="J46" s="8"/>
-      <c r="K46" s="8"/>
-      <c r="L46" s="8"/>
-      <c r="M46" s="8"/>
-      <c r="N46" s="8"/>
-      <c r="O46" s="8"/>
+      <c r="A46" s="3"/>
+      <c r="B46" s="4"/>
+      <c r="C46" s="4"/>
+      <c r="D46" s="4"/>
+      <c r="E46" s="4"/>
+      <c r="F46" s="4"/>
+      <c r="G46" s="4"/>
+      <c r="H46" s="4"/>
+      <c r="I46" s="4"/>
+      <c r="J46" s="4"/>
+      <c r="K46" s="4"/>
+      <c r="L46" s="4"/>
+      <c r="M46" s="4"/>
+      <c r="N46" s="4"/>
+      <c r="O46" s="4"/>
     </row>
   </sheetData>
   <mergeCells count="5">

</xml_diff>